<commit_message>
> (Off Topic) Update Prepare Framework File
+ It's now possible to add new sheet types automatically : "answers", "scores", "threats", "reference_controls" & "urn_prefix"
+ Removed useless localization for "copyright" field in "library_meta" sheet
</commit_message>
<xml_diff>
--- a/tools/prepare_framework_v2_config.xlsx
+++ b/tools/prepare_framework_v2_config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\misc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F116FD-F7B5-469C-A3B9-1A72900C8DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F258AEF-AEF3-40DE-914D-43AA73373CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{456AA15C-9F04-477A-B891-F9D422524496}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="120">
   <si>
     <t>urn_root</t>
   </si>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t>name</t>
-  </si>
-  <si>
-    <t>risk-framework_2025.example</t>
   </si>
   <si>
     <t>en</t>
@@ -87,9 +84,6 @@
 Designed for illustration and testing of the Excel generator.</t>
   </si>
   <si>
-    <t>© 2025 Example Organization</t>
-  </si>
-  <si>
     <t>intuitem</t>
   </si>
   <si>
@@ -105,9 +99,6 @@
     <t>Il s'agit d'un framework de démonstration.
 Il présente des exemples de règles, de contrôles et d'exigences.
 Il est conçu pour illustrer et tester le générateur Excel.</t>
-  </si>
-  <si>
-    <t>© 2025 Entreprise d'Exemple</t>
   </si>
   <si>
     <t>grp001</t>
@@ -570,6 +561,87 @@
   </si>
   <si>
     <t>my_framework.xlsx</t>
+  </si>
+  <si>
+    <t>base #3</t>
+  </si>
+  <si>
+    <t>base #4</t>
+  </si>
+  <si>
+    <t>base #5</t>
+  </si>
+  <si>
+    <t>base #6</t>
+  </si>
+  <si>
+    <t>base #7</t>
+  </si>
+  <si>
+    <t>answers_sheet_base_name</t>
+  </si>
+  <si>
+    <t>threats_sheet_base_name</t>
+  </si>
+  <si>
+    <t>reference_controls_sheet_base_name</t>
+  </si>
+  <si>
+    <t>urn_prefix_sheet_base_name</t>
+  </si>
+  <si>
+    <t>#answers_sheet_base_name</t>
+  </si>
+  <si>
+    <t>#threats_sheet_base_name</t>
+  </si>
+  <si>
+    <t>#reference_controls_sheet_base_name</t>
+  </si>
+  <si>
+    <t>#urn_prefix_sheet_base_name</t>
+  </si>
+  <si>
+    <t>answ</t>
+  </si>
+  <si>
+    <t>If you use it, sheets for "answers" will be created.</t>
+  </si>
+  <si>
+    <t>If you use it, sheets for "scores" will be created.</t>
+  </si>
+  <si>
+    <t>#scores_sheet_base_name</t>
+  </si>
+  <si>
+    <t>scores_sheet_base_name</t>
+  </si>
+  <si>
+    <t>scr</t>
+  </si>
+  <si>
+    <t>thrt</t>
+  </si>
+  <si>
+    <t>ref_ctrl</t>
+  </si>
+  <si>
+    <t>If you use it, sheets for "threats" will be created.</t>
+  </si>
+  <si>
+    <t>If you use it, sheets for "reference controls" will be created.</t>
+  </si>
+  <si>
+    <t>If you use it, sheets for "urn prefix" will be created.</t>
+  </si>
+  <si>
+    <t>urn_pref</t>
+  </si>
+  <si>
+    <t>risk-framework_2026.example</t>
+  </si>
+  <si>
+    <t>© 2026 Example Organization</t>
   </si>
 </sst>
 </file>
@@ -775,12 +847,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF5050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -809,8 +875,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB1A0C7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -968,36 +1040,47 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thick">
+      <right/>
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thick">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1051,7 +1134,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1080,16 +1163,108 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1101,15 +1276,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1119,86 +1285,14 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1256,6 +1350,7 @@
   </tableStyles>
   <colors>
     <mruColors>
+      <color rgb="FFB1A0C7"/>
       <color rgb="FFFF5050"/>
     </mruColors>
   </colors>
@@ -1271,11 +1366,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F507E4A3-5D6A-434A-B374-B18E54C9681D}" name="Tableau1" displayName="Tableau1" ref="A2:B1048576" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A2:B1048576" xr:uid="{F507E4A3-5D6A-434A-B374-B18E54C9681D}"/>
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F507E4A3-5D6A-434A-B374-B18E54C9681D}" name="Tableau1" displayName="Tableau1" ref="A2:G1048576" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A2:G1048576" xr:uid="{F507E4A3-5D6A-434A-B374-B18E54C9681D}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{87E32F60-8948-4823-9588-34007AFE9416}" name="base #1"/>
     <tableColumn id="2" xr3:uid="{A60015CC-AD6F-4FAD-B885-D8D6E2BB8DEF}" name="base #2"/>
+    <tableColumn id="3" xr3:uid="{59B3F822-630C-4835-A271-F082D160A4F6}" name="base #3"/>
+    <tableColumn id="4" xr3:uid="{DF576A64-64A9-43F4-98E5-A2C238F83308}" name="base #4"/>
+    <tableColumn id="5" xr3:uid="{751E47C5-0B0E-465A-9110-61A8D1F712DF}" name="base #5"/>
+    <tableColumn id="6" xr3:uid="{CBCF1460-F161-489C-BCAA-6155D645AB7D}" name="base #6"/>
+    <tableColumn id="7" xr3:uid="{EF1992F0-9AEC-45A3-8497-FB928E2ABCE5}" name="base #7"/>
   </tableColumns>
   <tableStyleInfo name="Style de tableau 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1611,360 +1711,378 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="64.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="56" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
+      <c r="I1" s="57"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
+      <c r="M1" s="58"/>
+    </row>
+    <row r="2" spans="1:13" ht="19.2" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="59" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="60"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="M2" s="61"/>
+    </row>
+    <row r="3" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="37"/>
+    </row>
+    <row r="4" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="43"/>
+    </row>
+    <row r="5" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="43"/>
+    </row>
+    <row r="6" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="46"/>
-    </row>
-    <row r="2" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="47" t="s">
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="42"/>
+      <c r="M6" s="43"/>
+    </row>
+    <row r="7" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="36"/>
+      <c r="L7" s="36"/>
+      <c r="M7" s="37"/>
+    </row>
+    <row r="8" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="44" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="46"/>
+      <c r="C8" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="42"/>
+      <c r="J8" s="42"/>
+      <c r="K8" s="42"/>
+      <c r="L8" s="42"/>
+      <c r="M8" s="43"/>
+    </row>
+    <row r="9" spans="1:13" ht="47.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="47" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="49"/>
+      <c r="C9" s="65" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="66"/>
+      <c r="L9" s="66"/>
+      <c r="M9" s="67"/>
+    </row>
+    <row r="10" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="47" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="49"/>
+      <c r="C10" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="42"/>
+      <c r="J10" s="42"/>
+      <c r="K10" s="42"/>
+      <c r="L10" s="42"/>
+      <c r="M10" s="43"/>
+    </row>
+    <row r="11" spans="1:13" ht="40.799999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="47" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="49"/>
+      <c r="C11" s="62" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
+      <c r="J11" s="63"/>
+      <c r="K11" s="63"/>
+      <c r="L11" s="63"/>
+      <c r="M11" s="64"/>
+    </row>
+    <row r="12" spans="1:13" s="3" customFormat="1" ht="46.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="32"/>
+      <c r="C12" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="49"/>
-    </row>
-    <row r="3" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="41" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="42"/>
-      <c r="L3" s="42"/>
-      <c r="M3" s="43"/>
-    </row>
-    <row r="4" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="50" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="34" t="s">
-        <v>60</v>
-      </c>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
-      <c r="K4" s="35"/>
-      <c r="L4" s="35"/>
-      <c r="M4" s="36"/>
-    </row>
-    <row r="5" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
+      <c r="M12" s="34"/>
+    </row>
+    <row r="13" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="36"/>
+      <c r="L13" s="36"/>
+      <c r="M13" s="37"/>
+    </row>
+    <row r="14" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="34" t="s">
+      <c r="B14" s="39"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" s="42"/>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="42"/>
+      <c r="L14" s="42"/>
+      <c r="M14" s="43"/>
+    </row>
+    <row r="15" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="42"/>
+      <c r="L15" s="42"/>
+      <c r="M15" s="43"/>
+    </row>
+    <row r="16" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="50" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="51"/>
+      <c r="C16" s="51"/>
+      <c r="D16" s="51"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="52"/>
+      <c r="G16" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="H16" s="42"/>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="42"/>
+      <c r="L16" s="42"/>
+      <c r="M16" s="43"/>
+    </row>
+    <row r="17" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="H5" s="35"/>
-      <c r="I5" s="35"/>
-      <c r="J5" s="35"/>
-      <c r="K5" s="35"/>
-      <c r="L5" s="35"/>
-      <c r="M5" s="36"/>
-    </row>
-    <row r="6" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="34" t="s">
-        <v>65</v>
-      </c>
-      <c r="H6" s="35"/>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="35"/>
-      <c r="M6" s="36"/>
-    </row>
-    <row r="7" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="41" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="42"/>
-      <c r="D7" s="42"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42"/>
-      <c r="G7" s="42"/>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="42"/>
-      <c r="M7" s="43"/>
-    </row>
-    <row r="8" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
-      <c r="K8" s="35"/>
-      <c r="L8" s="35"/>
-      <c r="M8" s="36"/>
-    </row>
-    <row r="9" spans="1:13" ht="47.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="37" t="s">
-        <v>83</v>
-      </c>
-      <c r="D9" s="38"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="38"/>
-      <c r="M9" s="39"/>
-    </row>
-    <row r="10" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35"/>
-      <c r="K10" s="35"/>
-      <c r="L10" s="35"/>
-      <c r="M10" s="36"/>
-    </row>
-    <row r="11" spans="1:13" ht="40.799999999999997" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="29" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="31" t="s">
+      <c r="B17" s="48"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="41" t="s">
+        <v>61</v>
+      </c>
+      <c r="H17" s="42"/>
+      <c r="I17" s="42"/>
+      <c r="J17" s="42"/>
+      <c r="K17" s="42"/>
+      <c r="L17" s="42"/>
+      <c r="M17" s="43"/>
+    </row>
+    <row r="18" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32"/>
-      <c r="K11" s="32"/>
-      <c r="L11" s="32"/>
-      <c r="M11" s="33"/>
-    </row>
-    <row r="12" spans="1:13" s="3" customFormat="1" ht="46.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="54" t="s">
+      <c r="B18" s="54"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" s="42"/>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="42"/>
+      <c r="L18" s="42"/>
+      <c r="M18" s="43"/>
+    </row>
+    <row r="19" spans="1:13" s="3" customFormat="1" ht="17.399999999999999" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19" s="32"/>
+      <c r="C19" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="54"/>
-      <c r="C12" s="55" t="s">
-        <v>69</v>
-      </c>
-      <c r="D12" s="56"/>
-      <c r="E12" s="56"/>
-      <c r="F12" s="56"/>
-      <c r="G12" s="56"/>
-      <c r="H12" s="56"/>
-      <c r="I12" s="56"/>
-      <c r="J12" s="56"/>
-      <c r="K12" s="56"/>
-      <c r="L12" s="56"/>
-      <c r="M12" s="56"/>
-    </row>
-    <row r="13" spans="1:13" ht="34.799999999999997" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="42"/>
-      <c r="L13" s="42"/>
-      <c r="M13" s="43"/>
-    </row>
-    <row r="14" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="50" t="s">
-        <v>56</v>
-      </c>
-      <c r="B14" s="51"/>
-      <c r="C14" s="51"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="34" t="s">
-        <v>62</v>
-      </c>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="35"/>
-      <c r="L14" s="35"/>
-      <c r="M14" s="36"/>
-    </row>
-    <row r="15" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="35"/>
-      <c r="L15" s="35"/>
-      <c r="M15" s="36"/>
-    </row>
-    <row r="16" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="57" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="58"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="58"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="34" t="s">
-        <v>89</v>
-      </c>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="35"/>
-      <c r="L16" s="35"/>
-      <c r="M16" s="36"/>
-    </row>
-    <row r="17" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="35"/>
-      <c r="L17" s="35"/>
-      <c r="M17" s="36"/>
-    </row>
-    <row r="18" spans="1:13" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="60" t="s">
-        <v>87</v>
-      </c>
-      <c r="B18" s="61"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="62"/>
-      <c r="G18" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="35"/>
-      <c r="L18" s="35"/>
-      <c r="M18" s="36"/>
-    </row>
-    <row r="19" spans="1:13" s="3" customFormat="1" ht="17.399999999999999" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="54" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="54"/>
-      <c r="C19" s="55" t="s">
-        <v>71</v>
-      </c>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="56"/>
-      <c r="J19" s="56"/>
-      <c r="K19" s="56"/>
-      <c r="L19" s="56"/>
-      <c r="M19" s="56"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
+      <c r="J19" s="34"/>
+      <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
+      <c r="M19" s="34"/>
     </row>
     <row r="20" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="33">
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:M11"/>
+    <mergeCell ref="C10:M10"/>
+    <mergeCell ref="C9:M9"/>
+    <mergeCell ref="C8:M8"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="G4:M4"/>
+    <mergeCell ref="G5:M5"/>
+    <mergeCell ref="G6:M6"/>
+    <mergeCell ref="A7:M7"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="C12:M12"/>
     <mergeCell ref="A19:B19"/>
@@ -1980,24 +2098,6 @@
     <mergeCell ref="G16:M16"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="G18:M18"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="G4:M4"/>
-    <mergeCell ref="G5:M5"/>
-    <mergeCell ref="G6:M6"/>
-    <mergeCell ref="A7:M7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:M11"/>
-    <mergeCell ref="C10:M10"/>
-    <mergeCell ref="C9:M9"/>
-    <mergeCell ref="C8:M8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2008,48 +2108,104 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.88671875" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" customWidth="1"/>
+    <col min="1" max="1" width="37.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="37.200000000000003" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
-        <v>91</v>
-      </c>
-      <c r="B1" s="64"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="37.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="68" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="70"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="26" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B2" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="26" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D2" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F3" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="G3" s="27" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -2062,30 +2218,30 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="70" customWidth="1"/>
-    <col min="3" max="3" width="121.44140625" customWidth="1"/>
+    <col min="3" max="3" width="129.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="29.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="65" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="66"/>
+      <c r="A1" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="31"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -2093,10 +2249,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2104,10 +2260,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -2115,10 +2271,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -2126,10 +2282,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2137,10 +2293,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2148,21 +2304,21 @@
         <v>6</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -2170,10 +2326,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -2181,21 +2337,76 @@
         <v>8</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>95</v>
+      <c r="A12" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>106</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>44</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="28" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2207,7 +2418,7 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{529A6840-0962-43F9-AA72-4A3CB85E552B}">
           <x14:formula1>
             <xm:f>_configs!$A$3:$A$4</xm:f>
@@ -2218,7 +2429,37 @@
           <x14:formula1>
             <xm:f>_configs!$B$3:$B$4</xm:f>
           </x14:formula1>
+          <xm:sqref>A17</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5EA7369B-4AB1-4D4B-989B-7334E4D68360}">
+          <x14:formula1>
+            <xm:f>_configs!$C$3:$C$4</xm:f>
+          </x14:formula1>
           <xm:sqref>A12</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EC5BEE9F-744F-463A-9F54-0EE3D0F27699}">
+          <x14:formula1>
+            <xm:f>_configs!$D$3:$D$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>A13</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0816A3FC-0403-484A-B88E-284465A372A0}">
+          <x14:formula1>
+            <xm:f>_configs!$E$3:$E$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>A14</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E972D39B-ABCA-4DFD-A4AA-9D63E2E5B130}">
+          <x14:formula1>
+            <xm:f>_configs!$F$3:$F$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>A15</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{90FE35AA-B224-4B4C-BAC9-54379286DCAA}">
+          <x14:formula1>
+            <xm:f>_configs!$G$3:$G$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>A16</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2244,19 +2485,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="67" t="s">
-        <v>72</v>
-      </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
+      <c r="A1" s="71" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
       <c r="E1" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -2271,43 +2512,43 @@
       </c>
       <c r="D2" s="14"/>
       <c r="E2" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="21" t="s">
-        <v>24</v>
-      </c>
       <c r="C3" s="21" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2325,7 +2566,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.109375" bestFit="1" customWidth="1"/>
@@ -2334,21 +2575,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="29.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="65" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="66"/>
+      <c r="A1" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="31"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="22" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -2356,21 +2597,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -2400,19 +2630,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="44.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="69" t="s">
-        <v>73</v>
-      </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
+      <c r="A1" s="73" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
       <c r="E1" s="10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -2426,43 +2656,43 @@
         <v>4</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="21" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C5" s="21"/>
     </row>

</xml_diff>